<commit_message>
feat: Improve train/test split
</commit_message>
<xml_diff>
--- a/data/excel/API properties.xlsx
+++ b/data/excel/API properties.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hioa365-my.sharepoint.com/personal/masun1863_oslomet_no/Documents/Dokumenter/ML Feature Properties/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="151" documentId="8_{0E741D0D-B1A2-46C0-8237-A963BC48DBDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1022ACD4-DD45-47FA-B771-ED84A37417E5}"/>
+  <xr:revisionPtr revIDLastSave="400" documentId="8_{0E741D0D-B1A2-46C0-8237-A963BC48DBDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{199F73AF-A72C-400F-A200-0EF5A0305818}"/>
   <bookViews>
-    <workbookView xWindow="13140" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{52E4DE00-B8E2-4867-A8EE-FA1EE720E88B}"/>
+    <workbookView xWindow="14130" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{52E4DE00-B8E2-4867-A8EE-FA1EE720E88B}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Complexity</t>
   </si>
@@ -153,13 +153,37 @@
   </si>
   <si>
     <t>Vinorelbine</t>
+  </si>
+  <si>
+    <t>LogP</t>
+  </si>
+  <si>
+    <t>Formal charge</t>
+  </si>
+  <si>
+    <t>Defined atom stereocenter count</t>
+  </si>
+  <si>
+    <t>Defined bond stereocenter count</t>
+  </si>
+  <si>
+    <t>Used data for Nartograstim for Granulocyte-Colony Stimulating factor</t>
+  </si>
+  <si>
+    <t>Data was collected from PubChem, and from ChemAxon via DrugBank for the compounds missing logP data in PubChem</t>
+  </si>
+  <si>
+    <t>Number of rings</t>
+  </si>
+  <si>
+    <t>All ring data was collected from DrugBank</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,8 +191,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,6 +209,30 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor theme="9" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -227,11 +281,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,46 +625,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23386EA2-7693-4D8A-BE8A-2E3E5D43DF0D}">
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.1796875" customWidth="1"/>
-    <col min="3" max="3" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -613,25 +691,37 @@
         <v>1144.4000000000001</v>
       </c>
       <c r="C2">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="D2">
         <v>10</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>22</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>9</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>76</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>495</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>2180</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>6</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -639,25 +729,40 @@
         <v>1620.7</v>
       </c>
       <c r="C3">
+        <v>-5.0999999999999996</v>
+      </c>
+      <c r="D3">
         <v>35</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>28</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>22</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>115</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>702</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>3480</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>13</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -665,25 +770,40 @@
         <v>129.16</v>
       </c>
       <c r="C4">
+        <v>-1.3</v>
+      </c>
+      <c r="D4">
         <v>2</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>1</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>3</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>9</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>91.5</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>132</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -691,25 +811,37 @@
         <v>4493</v>
       </c>
       <c r="C5">
+        <v>-18.3</v>
+      </c>
+      <c r="D5">
         <v>171</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>69</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>68</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>318</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>1890</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>10600</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>39</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -720,22 +852,37 @@
         <v>6</v>
       </c>
       <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
         <v>13</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>3</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>65</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>195</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>1760</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>15</v>
+      </c>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -743,25 +890,40 @@
         <v>161.4</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>-7.0000000000000007E-2</v>
       </c>
       <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
         <v>4</v>
       </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
       <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
         <v>6</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>88.6</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>62.2</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -769,25 +931,40 @@
         <v>748</v>
       </c>
       <c r="C8">
+        <v>3.2</v>
+      </c>
+      <c r="D8">
         <v>8</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>14</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>4</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>52</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>183</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>1190</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>18</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -795,51 +972,81 @@
         <v>543.5</v>
       </c>
       <c r="C9">
+        <v>1.3</v>
+      </c>
+      <c r="D9">
         <v>5</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>12</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>6</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>39</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>206</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>977</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>6</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
       <c r="B10">
         <v>384.2</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="5">
+        <v>1.53</v>
+      </c>
+      <c r="D10">
         <v>9</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>6</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>4</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>28</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>124</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>500</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>2</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -847,25 +1054,40 @@
         <v>381.4</v>
       </c>
       <c r="C11">
+        <v>3.4</v>
+      </c>
+      <c r="D11">
         <v>3</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>7</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>1</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>26</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>86.4</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>577</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -873,30 +1095,78 @@
         <v>778.9</v>
       </c>
       <c r="C12">
+        <v>3.6</v>
+      </c>
+      <c r="D12">
         <v>10</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>11</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>2</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>57</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>134</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>1690</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>8</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B13">
+        <v>942.1</v>
+      </c>
+      <c r="C13">
+        <v>-1.6</v>
+      </c>
+      <c r="D13">
+        <v>29</v>
+      </c>
+      <c r="E13">
+        <v>11</v>
+      </c>
+      <c r="F13">
+        <v>12</v>
+      </c>
+      <c r="G13">
+        <v>68</v>
+      </c>
+      <c r="H13">
+        <v>392</v>
+      </c>
+      <c r="I13">
+        <v>1820</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>6</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -904,30 +1174,72 @@
         <v>482.4</v>
       </c>
       <c r="C14">
+        <v>2.4</v>
+      </c>
+      <c r="D14">
         <v>4</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>10</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>5</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>35</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>155</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>750</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B15">
+        <v>623.70000000000005</v>
+      </c>
+      <c r="D15">
+        <v>13</v>
+      </c>
+      <c r="E15">
+        <v>18</v>
+      </c>
+      <c r="F15">
+        <v>12</v>
+      </c>
+      <c r="G15">
+        <v>43</v>
+      </c>
+      <c r="H15">
+        <v>374</v>
+      </c>
+      <c r="I15">
+        <v>519</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>4</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -935,25 +1247,40 @@
         <v>270.24</v>
       </c>
       <c r="C16">
+        <v>1.7</v>
+      </c>
+      <c r="D16">
         <v>1</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>5</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <v>3</v>
       </c>
-      <c r="F16">
+      <c r="G16">
         <v>20</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>87</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>410</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -961,30 +1288,45 @@
         <v>130.08000000000001</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>-0.9</v>
       </c>
       <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
         <v>3</v>
       </c>
-      <c r="E17">
+      <c r="F17">
         <v>2</v>
       </c>
-      <c r="F17">
+      <c r="G17">
         <v>9</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>58.2</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>199</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -992,25 +1334,40 @@
         <v>482.4</v>
       </c>
       <c r="C19">
+        <v>2.4</v>
+      </c>
+      <c r="D19">
         <v>4</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>10</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <v>5</v>
       </c>
-      <c r="F19">
+      <c r="G19">
         <v>35</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <v>155</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>750</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>4</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -1018,25 +1375,40 @@
         <v>368.4</v>
       </c>
       <c r="C20">
+        <v>3.2</v>
+      </c>
+      <c r="D20">
         <v>8</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>6</v>
       </c>
-      <c r="E20">
+      <c r="F20">
         <v>2</v>
       </c>
-      <c r="F20">
+      <c r="G20">
         <v>27</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <v>93.1</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>507</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>2</v>
+      </c>
+      <c r="M20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -1044,30 +1416,81 @@
         <v>1449.2</v>
       </c>
       <c r="C21">
+        <v>-2.6</v>
+      </c>
+      <c r="D21">
         <v>13</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>26</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <v>19</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <v>101</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>530</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>2960</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>18</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B22">
+        <v>146.13999999999999</v>
+      </c>
+      <c r="C22">
+        <v>-3.1</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>4</v>
+      </c>
+      <c r="F22">
+        <v>3</v>
+      </c>
+      <c r="G22">
+        <v>10</v>
+      </c>
+      <c r="H22">
+        <v>106</v>
+      </c>
+      <c r="I22">
+        <v>146</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>1</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -1075,25 +1498,40 @@
         <v>158.12</v>
       </c>
       <c r="C23">
+        <v>-2.2000000000000002</v>
+      </c>
+      <c r="D23">
         <v>1</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>3</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>4</v>
       </c>
-      <c r="F23">
+      <c r="G23">
         <v>11</v>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>113</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>225</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -1101,25 +1539,40 @@
         <v>204.29</v>
       </c>
       <c r="C24">
+        <v>1.8</v>
+      </c>
+      <c r="D24">
         <v>1</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>2</v>
       </c>
-      <c r="E24">
-        <v>0</v>
-      </c>
       <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
         <v>14</v>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>40.9</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>246</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>1</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -1127,25 +1580,40 @@
         <v>265.33</v>
       </c>
       <c r="C25">
+        <v>2.9</v>
+      </c>
+      <c r="D25">
         <v>5</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>4</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <v>2</v>
       </c>
-      <c r="F25">
+      <c r="G25">
         <v>18</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>92.3</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>290</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -1153,35 +1621,119 @@
         <v>554.6</v>
       </c>
       <c r="C26">
+        <v>-1.3</v>
+      </c>
+      <c r="D26">
         <v>8</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>13</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <v>4</v>
       </c>
-      <c r="F26">
+      <c r="G26">
         <v>36</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>288</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>1110</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>2</v>
+      </c>
+      <c r="L26">
+        <v>1</v>
+      </c>
+      <c r="M26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A27" s="6" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B27">
+        <v>727.8</v>
+      </c>
+      <c r="C27">
+        <v>-5.3</v>
+      </c>
+      <c r="D27">
+        <v>22</v>
+      </c>
+      <c r="E27">
+        <v>13</v>
+      </c>
+      <c r="F27">
+        <v>12</v>
+      </c>
+      <c r="G27">
+        <v>50</v>
+      </c>
+      <c r="H27">
+        <v>359</v>
+      </c>
+      <c r="I27">
+        <v>1170</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>7</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B28">
+        <v>1485.7</v>
+      </c>
+      <c r="C28" s="5">
+        <v>-4.4000000000000004</v>
+      </c>
+      <c r="D28">
+        <v>13</v>
+      </c>
+      <c r="E28">
+        <v>26</v>
+      </c>
+      <c r="F28">
+        <v>20</v>
+      </c>
+      <c r="G28">
+        <v>102</v>
+      </c>
+      <c r="H28">
+        <v>530</v>
+      </c>
+      <c r="I28">
+        <v>2960</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>18</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -1189,51 +1741,81 @@
         <v>272.25</v>
       </c>
       <c r="C29">
+        <v>2.4</v>
+      </c>
+      <c r="D29">
         <v>1</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>5</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <v>3</v>
       </c>
-      <c r="F29">
+      <c r="G29">
         <v>20</v>
       </c>
-      <c r="G29">
+      <c r="H29">
         <v>87</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>363</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="M29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>35</v>
       </c>
       <c r="B30">
         <v>785</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="5">
+        <v>2.44</v>
+      </c>
+      <c r="D30">
         <v>7</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>16</v>
       </c>
-      <c r="E30">
+      <c r="F30">
         <v>7</v>
       </c>
-      <c r="F30">
+      <c r="G30">
         <v>54</v>
       </c>
-      <c r="G30">
+      <c r="H30">
         <v>182</v>
       </c>
-      <c r="H30">
+      <c r="I30">
         <v>1150</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>18</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -1241,25 +1823,40 @@
         <v>720.9</v>
       </c>
       <c r="C31">
+        <v>6</v>
+      </c>
+      <c r="D31">
         <v>18</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <v>9</v>
       </c>
-      <c r="E31">
+      <c r="F31">
         <v>4</v>
       </c>
-      <c r="F31">
+      <c r="G31">
         <v>50</v>
       </c>
-      <c r="G31">
+      <c r="H31">
         <v>202</v>
       </c>
-      <c r="H31">
+      <c r="I31">
         <v>1040</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
+        <v>0</v>
+      </c>
+      <c r="M31">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -1267,23 +1864,57 @@
         <v>3354.1</v>
       </c>
       <c r="C32">
+        <v>-6.1</v>
+      </c>
+      <c r="D32">
         <v>67</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <v>50</v>
       </c>
-      <c r="E32">
+      <c r="F32">
         <v>41</v>
       </c>
-      <c r="F32">
+      <c r="G32">
         <v>229</v>
       </c>
-      <c r="G32">
+      <c r="H32">
         <v>1390</v>
       </c>
-      <c r="H32">
+      <c r="I32">
         <v>7840</v>
       </c>
+      <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
+      <c r="L32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B36" s="8"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1291,6 +1922,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="b4431929-4c33-46cd-93fc-96c7645c6ebe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100014AE37F2444474EA4D68E839ECCDDD3" ma:contentTypeVersion="10" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="264f9428646d58ecbe2ecf52a3651c39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="b4431929-4c33-46cd-93fc-96c7645c6ebe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1935da1053663dbc7bdeb9684e1c7118" ns3:_="">
     <xsd:import namespace="b4431929-4c33-46cd-93fc-96c7645c6ebe"/>
@@ -1472,24 +2120,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69D1889B-9597-4DC1-A6DD-7013C54D4562}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="b4431929-4c33-46cd-93fc-96c7645c6ebe"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="b4431929-4c33-46cd-93fc-96c7645c6ebe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E1EB5A0-0F25-45C1-BF1C-C4B740B60E41}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89988FEA-A84F-4B0D-A80E-275F13FBDA1C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1507,30 +2162,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E1EB5A0-0F25-45C1-BF1C-C4B740B60E41}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69D1889B-9597-4DC1-A6DD-7013C54D4562}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="b4431929-4c33-46cd-93fc-96c7645c6ebe"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{fec81f12-6286-4550-8911-f446fcdafa1f}" enabled="0" method="" siteId="{fec81f12-6286-4550-8911-f446fcdafa1f}" removed="1"/>

</xml_diff>